<commit_message>
Foundational Code block for Registration App
</commit_message>
<xml_diff>
--- a/Lead Upload Test Data.xlsx
+++ b/Lead Upload Test Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rhod_\Documents\StudyLinkLeadQualification\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CC1956C-057A-463F-91DA-495AAFD8DAEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87ACA507-FE5A-42DE-8BB4-AB60B2762185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,117 +58,78 @@
     <t>Database Purchase</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-001</t>
-  </si>
-  <si>
     <t>Bui Gia Vy</t>
   </si>
   <si>
     <t>upload001@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-002</t>
-  </si>
-  <si>
     <t>Le Thi Nam</t>
   </si>
   <si>
     <t>upload002@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-003</t>
-  </si>
-  <si>
     <t>Le Anh An</t>
   </si>
   <si>
     <t>upload003@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-004</t>
-  </si>
-  <si>
     <t>Vo Ngoc Quyen</t>
   </si>
   <si>
     <t>upload004@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-005</t>
-  </si>
-  <si>
     <t>Dang Gia Yen</t>
   </si>
   <si>
     <t>upload005@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-006</t>
-  </si>
-  <si>
     <t>Tran Duc Binh</t>
   </si>
   <si>
     <t>upload006@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-007</t>
-  </si>
-  <si>
     <t>Dang Duc Mai</t>
   </si>
   <si>
     <t>upload007@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-008</t>
-  </si>
-  <si>
     <t>Dang Thi Chi</t>
   </si>
   <si>
     <t>upload008@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-009</t>
-  </si>
-  <si>
     <t>Bui Gia Dung</t>
   </si>
   <si>
     <t>upload009@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-010</t>
-  </si>
-  <si>
     <t>Ngo Hong Yen</t>
   </si>
   <si>
     <t>upload010@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-011</t>
-  </si>
-  <si>
     <t>Pham Ngoc Hieu</t>
   </si>
   <si>
     <t>upload011@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-012</t>
-  </si>
-  <si>
     <t>Ngo Quang An</t>
   </si>
   <si>
     <t>upload012@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-013</t>
-  </si>
-  <si>
     <t>Le Duc Chi</t>
   </si>
   <si>
@@ -178,108 +139,72 @@
     <t>Ho Chi Minh City</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-014</t>
-  </si>
-  <si>
     <t>Dang Ngoc Quyen</t>
   </si>
   <si>
     <t>upload014@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-015</t>
-  </si>
-  <si>
     <t>Dang Hong Mai</t>
   </si>
   <si>
     <t>upload015@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-016</t>
-  </si>
-  <si>
     <t>Do Anh Quyen</t>
   </si>
   <si>
     <t>upload016@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-017</t>
-  </si>
-  <si>
     <t>Pham Van An</t>
   </si>
   <si>
     <t>upload017@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-018</t>
-  </si>
-  <si>
     <t>Bui Thanh Son</t>
   </si>
   <si>
     <t>upload018@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-019</t>
-  </si>
-  <si>
     <t>Nguyen Van Quyen</t>
   </si>
   <si>
     <t>upload019@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-020</t>
-  </si>
-  <si>
     <t>Do Thanh Tam</t>
   </si>
   <si>
     <t>upload020@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-021</t>
-  </si>
-  <si>
     <t>Bui Anh An</t>
   </si>
   <si>
     <t>upload021@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-022</t>
-  </si>
-  <si>
     <t>Tran Hong Yen</t>
   </si>
   <si>
     <t>upload022@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-023</t>
-  </si>
-  <si>
     <t>Do Gia An</t>
   </si>
   <si>
     <t>upload023@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-024</t>
-  </si>
-  <si>
     <t>Bui Hong Yen</t>
   </si>
   <si>
     <t>upload024@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-025</t>
-  </si>
-  <si>
     <t>Bui Ngoc Yen</t>
   </si>
   <si>
@@ -289,49 +214,124 @@
     <t>Hanoi</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-026</t>
-  </si>
-  <si>
     <t>Pham Anh Yen</t>
   </si>
   <si>
     <t>upload026@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-027</t>
-  </si>
-  <si>
     <t>upload027@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-028</t>
-  </si>
-  <si>
     <t>Bui Thanh Binh</t>
   </si>
   <si>
     <t>upload028@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-029</t>
-  </si>
-  <si>
     <t>Nguyen Minh Mai</t>
   </si>
   <si>
     <t>upload029@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-030</t>
-  </si>
-  <si>
     <t>Tran Gia Son</t>
   </si>
   <si>
     <t>upload030@example.com</t>
   </si>
   <si>
-    <t>TEST-UPLOAD-031</t>
+    <t>TEST-UPLOAD-131</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-101</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-102</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-103</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-104</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-105</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-106</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-107</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-108</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-109</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-110</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-111</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-112</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-113</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-114</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-115</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-116</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-117</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-118</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-119</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-120</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-121</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-122</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-123</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-124</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-125</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-126</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-127</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-128</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-129</t>
+  </si>
+  <si>
+    <t>TEST-UPLOAD-130</t>
   </si>
 </sst>
 </file>
@@ -709,18 +709,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G32"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="15.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.6875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.4375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.5625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.3125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.25" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.3125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.8125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -743,9 +743,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
-        <v>103</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -766,18 +766,18 @@
         <v>2006</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" t="s">
         <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
       </c>
       <c r="C3">
         <v>977893287</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
         <v>10</v>
@@ -789,18 +789,18 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C4">
         <v>942180967</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
@@ -812,18 +812,18 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C5">
         <v>981003390</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
@@ -835,18 +835,18 @@
         <v>2007</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C6">
         <v>938347017</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E6" t="s">
         <v>10</v>
@@ -858,18 +858,18 @@
         <v>2006</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>78</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C7">
         <v>914538401</v>
       </c>
       <c r="D7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
@@ -881,18 +881,18 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>79</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C8">
         <v>946100330</v>
       </c>
       <c r="D8" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="E8" t="s">
         <v>10</v>
@@ -904,18 +904,18 @@
         <v>2007</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C9">
         <v>919345145</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E9" t="s">
         <v>10</v>
@@ -927,18 +927,18 @@
         <v>2004</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>81</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="C10">
         <v>931007728</v>
       </c>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
@@ -950,18 +950,18 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>82</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="C11">
         <v>926616630</v>
       </c>
       <c r="D11" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -973,18 +973,18 @@
         <v>2006</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A12" t="s">
-        <v>39</v>
+        <v>83</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C12">
         <v>903269910</v>
       </c>
       <c r="D12" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -996,21 +996,21 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>84</v>
       </c>
       <c r="B13" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="C13">
         <v>909546111</v>
       </c>
       <c r="D13" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="E13" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="F13" t="s">
         <v>11</v>
@@ -1019,18 +1019,18 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="C14">
         <v>995597297</v>
       </c>
       <c r="D14" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -1042,21 +1042,21 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>86</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="C15">
         <v>924393328</v>
       </c>
       <c r="D15" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="E15" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="F15" t="s">
         <v>11</v>
@@ -1065,21 +1065,21 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A16" t="s">
-        <v>52</v>
+        <v>87</v>
       </c>
       <c r="B16" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="C16">
         <v>916011084</v>
       </c>
       <c r="D16" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="E16" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="F16" t="s">
         <v>11</v>
@@ -1088,21 +1088,21 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A17" t="s">
-        <v>55</v>
+        <v>88</v>
       </c>
       <c r="B17" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="C17">
         <v>997482123</v>
       </c>
       <c r="D17" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="E17" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="F17" t="s">
         <v>11</v>
@@ -1111,21 +1111,21 @@
         <v>2007</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A18" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B18" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="C18">
         <v>914330146</v>
       </c>
       <c r="D18" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="E18" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="F18" t="s">
         <v>11</v>
@@ -1134,21 +1134,21 @@
         <v>2007</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A19" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="B19" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="C19">
         <v>924589215</v>
       </c>
       <c r="D19" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="E19" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="F19" t="s">
         <v>11</v>
@@ -1157,21 +1157,21 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A20" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
       <c r="B20" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="C20">
         <v>989290075</v>
       </c>
       <c r="D20" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="E20" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="F20" t="s">
         <v>11</v>
@@ -1180,21 +1180,21 @@
         <v>2006</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A21" t="s">
-        <v>67</v>
+        <v>92</v>
       </c>
       <c r="B21" t="s">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="C21">
         <v>917145211</v>
       </c>
       <c r="D21" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="E21" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="F21" t="s">
         <v>11</v>
@@ -1203,21 +1203,21 @@
         <v>2007</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A22" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="B22" t="s">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="C22">
         <v>902551716</v>
       </c>
       <c r="D22" t="s">
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="E22" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="F22" t="s">
         <v>11</v>
@@ -1226,21 +1226,21 @@
         <v>2004</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>94</v>
       </c>
       <c r="B23" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="C23">
         <v>996690911</v>
       </c>
       <c r="D23" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="E23" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="F23" t="s">
         <v>11</v>
@@ -1249,21 +1249,21 @@
         <v>2004</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A24" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="B24" t="s">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="C24">
         <v>965697778</v>
       </c>
       <c r="D24" t="s">
-        <v>78</v>
+        <v>56</v>
       </c>
       <c r="E24" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="F24" t="s">
         <v>11</v>
@@ -1272,21 +1272,21 @@
         <v>2004</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A25" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="B25" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="C25">
         <v>949170317</v>
       </c>
       <c r="D25" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="E25" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="F25" t="s">
         <v>11</v>
@@ -1295,21 +1295,21 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A26" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="B26" t="s">
-        <v>83</v>
+        <v>59</v>
       </c>
       <c r="C26">
         <v>905429382</v>
       </c>
       <c r="D26" t="s">
-        <v>84</v>
+        <v>60</v>
       </c>
       <c r="E26" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="F26" t="s">
         <v>11</v>
@@ -1318,21 +1318,21 @@
         <v>2006</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A27" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="B27" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="C27">
         <v>935643633</v>
       </c>
       <c r="D27" t="s">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="E27" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="F27" t="s">
         <v>11</v>
@@ -1341,21 +1341,21 @@
         <v>2007</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A28" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="B28" t="s">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="C28">
         <v>953227501</v>
       </c>
       <c r="D28" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="E28" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="F28" t="s">
         <v>11</v>
@@ -1364,21 +1364,21 @@
         <v>2006</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A29" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="B29" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C29">
         <v>974366875</v>
       </c>
       <c r="D29" t="s">
-        <v>93</v>
+        <v>66</v>
       </c>
       <c r="E29" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="F29" t="s">
         <v>11</v>
@@ -1387,21 +1387,21 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A30" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="B30" t="s">
-        <v>95</v>
+        <v>67</v>
       </c>
       <c r="C30">
         <v>904904954</v>
       </c>
       <c r="D30" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="E30" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="F30" t="s">
         <v>11</v>
@@ -1410,21 +1410,21 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A31" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B31" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="C31">
         <v>973043201</v>
       </c>
       <c r="D31" t="s">
-        <v>99</v>
+        <v>70</v>
       </c>
       <c r="E31" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="F31" t="s">
         <v>11</v>
@@ -1433,21 +1433,21 @@
         <v>2007</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A32" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B32" t="s">
-        <v>101</v>
+        <v>71</v>
       </c>
       <c r="C32">
         <v>951337420</v>
       </c>
       <c r="D32" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
       <c r="E32" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="F32" t="s">
         <v>11</v>

</xml_diff>